<commit_message>
Complete initial iteration of data visualization graphs
- Finalized chart generation functionality for calculated financial data

- Finished dashboard layout with Streamlit components and proper styling

The visualization system is now fully functional, reading configuration from
visualizations_map.json, processing financial data from Excel sources, and
generating interactive charts to display financing sources across different
models and scenarios.
</commit_message>
<xml_diff>
--- a/backend/Rwanda/financial-statements-Aligned.xlsx
+++ b/backend/Rwanda/financial-statements-Aligned.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/Rwanda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_0C7E6E461F42155A05CCE6F1FD8A6A735C001098" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9669516B-9363-40A9-8AC7-F1E890592AAA}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_0C7E6E461F42155A05CCE6F1FD8A6A735C001098" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76E173EE-C051-4A68-B36A-D16FA202389A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity (Only E-Cooking)" sheetId="1" r:id="rId1"/>
@@ -17955,40 +17955,40 @@
         <v>5</v>
       </c>
       <c r="D25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="F25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="G25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="H25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="I25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="J25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="K25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="L25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="M25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="N25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="O25" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:15" ht="15.5" x14ac:dyDescent="0.35">
@@ -19647,40 +19647,40 @@
         <v>5</v>
       </c>
       <c r="D61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="E61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="F61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="G61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="H61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="I61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="J61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="K61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="L61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="M61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="N61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="O61" s="18">
-        <v>0</v>
+        <v>123</v>
       </c>
     </row>
     <row r="62" spans="1:15" ht="15.5" x14ac:dyDescent="0.35">

</xml_diff>